<commit_message>
docs: align 0.7.1 candidate review state
</commit_message>
<xml_diff>
--- a/docs/audits/ElastOS-Home-Journey-Audit.xlsx
+++ b/docs/audits/ElastOS-Home-Journey-Audit.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="1" r:id="R9c6a3bc57b884a64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journey Matrix" sheetId="2" r:id="Ra58375695461449f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Index" sheetId="3" r:id="R2de9f38624804747"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="4" r:id="Re76454159b5941a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prioritized Plan" sheetId="5" r:id="R834deeb1cdba4301"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me + Evidence" sheetId="6" r:id="Rc1d41e9b1ab5410c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Principles Review" sheetId="7" r:id="Rb48e61790ac64467"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="1" r:id="R3750605e5f55415a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journey Matrix" sheetId="2" r:id="R41094babc9824b7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Index" sheetId="3" r:id="R2c6710fdd154464c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="4" r:id="R10c8b7c453fb44b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prioritized Plan" sheetId="5" r:id="R6fbcb4f0c7d24123"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me + Evidence" sheetId="6" r:id="R8db7feecbd184105"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Principles Review" sheetId="7" r:id="R92334268b0c04985"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -683,7 +683,7 @@
         <x:color rgb="FF226443"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F1E8"/>
         </x:patternFill>
       </x:fill>
@@ -694,7 +694,7 @@
         <x:color rgb="FF315D8C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FF"/>
         </x:patternFill>
       </x:fill>
@@ -705,7 +705,7 @@
         <x:color rgb="FF983F37"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE9E7"/>
         </x:patternFill>
       </x:fill>
@@ -716,7 +716,7 @@
         <x:color rgb="FF805711"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0D4"/>
         </x:patternFill>
       </x:fill>
@@ -727,7 +727,7 @@
         <x:color rgb="FF805711"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0D4"/>
         </x:patternFill>
       </x:fill>
@@ -738,7 +738,7 @@
         <x:color rgb="FF4D5664"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEFF0F2"/>
         </x:patternFill>
       </x:fill>
@@ -749,7 +749,7 @@
         <x:color rgb="FF4D5664"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEFF0F2"/>
         </x:patternFill>
       </x:fill>
@@ -760,7 +760,7 @@
         <x:color rgb="FF805711"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0D4"/>
         </x:patternFill>
       </x:fill>
@@ -1172,22 +1172,22 @@
     </x:row>
     <x:row r="2" ht="16.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | Mapped source does not mean tested product. Live outcomes and static control coverage are counted independently.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | Source coverage and observed product behavior remain separate measures.</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | Mapped source does not mean tested product. Live outcomes and static control coverage are counted independently.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | Source coverage and observed product behavior remain separate measures.</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | Mapped source does not mean tested product. Live outcomes and static control coverage are counted independently.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | Source coverage and observed product behavior remain separate measures.</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | Mapped source does not mean tested product. Live outcomes and static control coverage are counted independently.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | Source coverage and observed product behavior remain separate measures.</x:v>
       </x:c>
       <x:c r="E2" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | Mapped source does not mean tested product. Live outcomes and static control coverage are counted independently.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | Source coverage and observed product behavior remain separate measures.</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | Mapped source does not mean tested product. Live outcomes and static control coverage are counted independently.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | Source coverage and observed product behavior remain separate measures.</x:v>
       </x:c>
       <x:c r="G2" s="3"/>
       <x:c r="H2" s="3"/>
@@ -1197,22 +1197,22 @@
     </x:row>
     <x:row r="3" ht="16.5" customHeight="1">
       <x:c r="A3" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | Mapped source does not mean tested product. Live outcomes and static control coverage are counted independently.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | Source coverage and observed product behavior remain separate measures.</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | Mapped source does not mean tested product. Live outcomes and static control coverage are counted independently.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | Source coverage and observed product behavior remain separate measures.</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | Mapped source does not mean tested product. Live outcomes and static control coverage are counted independently.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | Source coverage and observed product behavior remain separate measures.</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | Mapped source does not mean tested product. Live outcomes and static control coverage are counted independently.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | Source coverage and observed product behavior remain separate measures.</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | Mapped source does not mean tested product. Live outcomes and static control coverage are counted independently.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | Source coverage and observed product behavior remain separate measures.</x:v>
       </x:c>
       <x:c r="F3" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | Mapped source does not mean tested product. Live outcomes and static control coverage are counted independently.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | Source coverage and observed product behavior remain separate measures.</x:v>
       </x:c>
       <x:c r="G3" s="3"/>
       <x:c r="H3" s="3"/>
@@ -3131,7 +3131,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a302113bfe44b03"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50c9a5ba1c38444f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3984,7 +3984,7 @@
         <x:v>Catalog items retain names/icons, keyboard focus, and honest no-result state.</x:v>
       </x:c>
       <x:c r="F16" s="12" t="str">
-        <x:v>Launcher browsing retains 16 named apps; grid/list and Escape/focus return pass (E-033). Matching/absent search passes through the separate toolbar Search surface at 2e9644d2 (E-037). Launcher itself is intentionally browse-only.</x:v>
+        <x:v>Launcher browsing exposes 16 named apps. Grid/list, Search, Escape, and focus return have prior live proof. E-108 confirms that every current launcher target opens through Home search on the isolated candidate install.</x:v>
       </x:c>
       <x:c r="G16" s="3" t="str">
         <x:v>safe-read-only</x:v>
@@ -4007,7 +4007,7 @@
       <x:c r="L16" s="3" t="str"/>
       <x:c r="M16" s="3" t="str"/>
       <x:c r="N16" s="3" t="str">
-        <x:v>E-033; E-037</x:v>
+        <x:v>E-033; E-037; E-108</x:v>
       </x:c>
       <x:c r="O16" s="3" t="str">
         <x:v>S-010</x:v>
@@ -7382,7 +7382,7 @@
         <x:v>Runtime validates names/ownership; failures leave no ambiguous duplicate.</x:v>
       </x:c>
       <x:c r="F68" s="12" t="str">
-        <x:v>Audit folder and fixture creation pass. F25 invalid-name→corrected-name retry now creates exactly one audit-retry-verified folder; generic guidance remains open. F26 current Runtime/UI sends create_only but installed object-provider rejects that unknown field. Original70B audit file is preserved; provider-specific install pending. E067freshobjectprovider fixes create-only: existingauditau.md70Bpreserved, collisionclear, correctednamecreatesonefile. F25/F48guidance/a11ygapsstay.</x:v>
+        <x:v>Audit folder and fixture creation pass. Corrected-name retry creates exactly one item. Runtime create-only protection preserves an existing file and reports collisions clearly. E-108 confirms the current managed Runtime selects the installed object-provider; remaining guidance and accessibility work stay tracked by F-25 and F-48.</x:v>
       </x:c>
       <x:c r="G68" s="3" t="str">
         <x:v>controlled-files</x:v>
@@ -7405,7 +7405,7 @@
       </x:c>
       <x:c r="M68" s="3" t="str"/>
       <x:c r="N68" s="3" t="str">
-        <x:v>E-044; E-059; E-067</x:v>
+        <x:v>E-044; E-059; E-067; E-108</x:v>
       </x:c>
       <x:c r="O68" s="3" t="str">
         <x:v>S-060, S-061</x:v>
@@ -13540,13 +13540,13 @@
         <x:v>Runtime can start the provider through the shared Init contract, confirm readiness and read offers.</x:v>
       </x:c>
       <x:c r="F163" s="12" t="str">
-        <x:v>Independent Runtime Init envelope config and process tests pass (2/2). Built release and installed model-provider match SHA435701d7...; installed manifest verifies. Actual Assistant reaches truthful zero-offer state. Configuration still contains no execution offers.</x:v>
+        <x:v>The installed candidate starts model-provider through the shared Init contract and confirms readiness. The release and installed provider artifacts match. Assistant reaches the truthful zero-offer state; one approved compatible offer is the next setup requirement.</x:v>
       </x:c>
       <x:c r="G163" s="3" t="str">
         <x:v>safe-read-only</x:v>
       </x:c>
       <x:c r="H163" s="3" t="str">
-        <x:v>source-defect</x:v>
+        <x:v>implemented-config-gated</x:v>
       </x:c>
       <x:c r="I163" s="3" t="str">
         <x:v>Background Init/readiness; no app control</x:v>
@@ -13564,7 +13564,7 @@
         <x:v>Prior startup log reported model-provider startup failed; source shows incompatible normal Init envelope. [Prior bounded startup finding; no new provider execution/test in this audit.]</x:v>
       </x:c>
       <x:c r="N163" s="3" t="str">
-        <x:v>E-036; E-039; E-054</x:v>
+        <x:v>E-036; E-039; E-054; E-108</x:v>
       </x:c>
       <x:c r="O163" s="3" t="str">
         <x:v>S-154, S-155, S-156</x:v>
@@ -13589,7 +13589,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="U163" s="3" t="str">
-        <x:v>Current normal Init serializes fields rejected by the strict model config. Startup repair and process proof remain open.</x:v>
+        <x:v>The provider lifecycle is installed and healthy. Model execution begins after an operator selects and configures an approved offer.</x:v>
       </x:c>
     </x:row>
     <x:row r="164" ht="153" customHeight="1">
@@ -13698,7 +13698,7 @@
       </x:c>
       <x:c r="M165" s="3" t="str"/>
       <x:c r="N165" s="3" t="str">
-        <x:v>E-036; E-039</x:v>
+        <x:v>E-036; E-039; E-108</x:v>
       </x:c>
       <x:c r="O165" s="3" t="str">
         <x:v>S-160, S-159</x:v>
@@ -13723,7 +13723,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="U165" s="3" t="str">
-        <x:v>Missing config is a valid zero-offer state. Invalid config or the current Init failure is separate; useful guidance still needs live review.</x:v>
+        <x:v>Missing configuration is a valid zero-offer state. Invalid configuration remains a separate failure branch; useful setup guidance still needs live review.</x:v>
       </x:c>
     </x:row>
     <x:row r="166" ht="153" customHeight="1">
@@ -13947,7 +13947,7 @@
         <x:v>Runtime admits page and engine; unavailable engine/network is explicit rather than a blank success.</x:v>
       </x:c>
       <x:c r="F169" s="12" t="str">
-        <x:v>First ela.city page reached Ready through MicroVM after34.4s. After recovery from a native-confirm automation stall, a new audit Home tab failed default ela.city and example.com startup with bounded closed-effects message. F-43. Current6edc667b retest: cold initial page renders; subsequent navigation delivers Example Domain frame but session fails, and one clean app reopen fails immediately. F43 remains open. E064 foreground retest successfully launches, navigates, closes and reopens. Retain earlier background/intermittent F43; full cleanup and controlled expiry remain unproved.</x:v>
+        <x:v>Earlier foreground runs found intermittent startup and navigation failures. E-108 adds a current cold launch: the macOS VM path reached Ready in 38.5 seconds, then Home Close removed the VM supervisor, VZ supervisor, and TURN process. The older intermittent finding remains open until repeated navigation and restart acceptance passes.</x:v>
       </x:c>
       <x:c r="G169" s="3" t="str">
         <x:v>controlled-network</x:v>
@@ -13970,7 +13970,7 @@
       </x:c>
       <x:c r="M169" s="3" t="str"/>
       <x:c r="N169" s="3" t="str">
-        <x:v>E-053; E-060; E-064</x:v>
+        <x:v>E-053; E-060; E-064; E-108</x:v>
       </x:c>
       <x:c r="O169" s="3" t="str">
         <x:v>S-163</x:v>
@@ -15719,7 +15719,7 @@
         <x:v>Runtime owns principal, typed resources and provider selection. Installed manifests alone do not prove provider health.</x:v>
       </x:c>
       <x:c r="F196" s="12" t="str">
-        <x:v>Exact installed localhost/did/object/content-block-graph manifests verify. Authenticated Home and bounded audit-file lifecycle prove useful local operations; full identity/rights/provider-negative coverage requires isolated fixtures.</x:v>
+        <x:v>The isolated candidate registers the local identity, object, and content providers in both gateway and managed Runtime paths. Authenticated Home, Library content visibility, create-only behavior, and all launcher targets provide current useful proof; negative provider and rights cases still need controlled fixtures.</x:v>
       </x:c>
       <x:c r="G196" s="3" t="str">
         <x:v>safe-read-only</x:v>
@@ -15739,7 +15739,7 @@
       <x:c r="L196" s="3" t="str"/>
       <x:c r="M196" s="3" t="str"/>
       <x:c r="N196" s="3" t="str">
-        <x:v>E-043; E-051; E-054</x:v>
+        <x:v>E-043; E-051; E-054; E-108</x:v>
       </x:c>
       <x:c r="O196" s="3" t="str">
         <x:v>S-183</x:v>
@@ -16114,7 +16114,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc857206eb4214faf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R562c5740ef324d73"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27775,8 +27775,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfaf5f73df17346f3"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra26f2f807e3e46ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7017081ee9e147bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d7f30e34d784a20"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27995,22 +27995,22 @@
         <x:v>source-contract-bug</x:v>
       </x:c>
       <x:c r="E8" s="3" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Fixed and installed-verified</x:v>
       </x:c>
       <x:c r="F8" s="3" t="str">
-        <x:v>prior startup warning plus source-confirmed envelope mismatch</x:v>
+        <x:v>Focused source tests plus isolated installed candidate proof</x:v>
       </x:c>
       <x:c r="G8" s="3" t="str">
-        <x:v>Assistant cannot reach even the valid zero-offer state through this failed provider startup. Adding model offers alone does not repair the envelope.</x:v>
+        <x:v>Assistant reaches the valid zero-offer state. Model execution begins after an approved compatible offer is configured.</x:v>
       </x:c>
       <x:c r="H8" s="3" t="str">
-        <x:v>Runtime ProviderConfig serializes allowed_paths, read_only and encryption_key. Model BridgeProviderConfig denies unknown fields and declares only base_path and extra, so normal Init deserialization rejects the shared envelope.</x:v>
+        <x:v>The old model parser accepted fewer fields than Runtime's shared Init envelope.</x:v>
       </x:c>
       <x:c r="I8" s="3" t="str">
-        <x:v>Align the exact existing bridge Init contract in its owning provider parser while preserving strict validation; keep the single provider lifecycle.</x:v>
+        <x:v>Keep the shared Init contract and strict offer validation in regression coverage.</x:v>
       </x:c>
       <x:c r="J8" s="3" t="str">
-        <x:v>Serialize the real Runtime ProviderConfig and pass it through the model process Init/status path with zero offers; require correct identity/readiness and bounded failure on invalid fields.</x:v>
+        <x:v>Runtime Init, readiness, and Assistant zero-offer behavior pass with matching installed artifacts.</x:v>
       </x:c>
       <x:c r="K8" s="3" t="str">
         <x:v>MODEL-01; AI-04</x:v>
@@ -30287,7 +30287,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R812f9edd395e47b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d6ceee7dd914057"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32414,7 +32414,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fb514e071b940f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14d89847794342f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32465,22 +32465,22 @@
     </x:row>
     <x:row r="2" ht="16.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | This workbook separates what source defines from what a person actually tested.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | This workbook separates source coverage from observed product behavior.</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | This workbook separates what source defines from what a person actually tested.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | This workbook separates source coverage from observed product behavior.</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | This workbook separates what source defines from what a person actually tested.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | This workbook separates source coverage from observed product behavior.</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | This workbook separates what source defines from what a person actually tested.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | This workbook separates source coverage from observed product behavior.</x:v>
       </x:c>
       <x:c r="E2" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | This workbook separates what source defines from what a person actually tested.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | This workbook separates source coverage from observed product behavior.</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | This workbook separates what source defines from what a person actually tested.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | This workbook separates source coverage from observed product behavior.</x:v>
       </x:c>
       <x:c r="G2" s="3"/>
       <x:c r="H2" s="3"/>
@@ -32491,22 +32491,22 @@
     </x:row>
     <x:row r="3" ht="16.5" customHeight="1">
       <x:c r="A3" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | This workbook separates what source defines from what a person actually tested.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | This workbook separates source coverage from observed product behavior.</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | This workbook separates what source defines from what a person actually tested.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | This workbook separates source coverage from observed product behavior.</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | This workbook separates what source defines from what a person actually tested.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | This workbook separates source coverage from observed product behavior.</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | This workbook separates what source defines from what a person actually tested.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | This workbook separates source coverage from observed product behavior.</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | This workbook separates what source defines from what a person actually tested.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | This workbook separates source coverage from observed product behavior.</x:v>
       </x:c>
       <x:c r="F3" s="9" t="str">
-        <x:v>PARTIAL LIVE AUDIT / BASELINE | This workbook separates what source defines from what a person actually tested.</x:v>
+        <x:v>CURRENT INSTALLED AUDIT | This workbook separates source coverage from observed product behavior.</x:v>
       </x:c>
       <x:c r="G3" s="3"/>
       <x:c r="H3" s="3"/>
@@ -32571,16 +32571,16 @@
         <x:v>Source</x:v>
       </x:c>
       <x:c r="C6" s="23" t="str">
-        <x:v>feat/protected-content-uiux-reconstruction @ 8e5eb88b8ec566a9ff3261efa84e1fc9a6b1f5c3 | tree 584f59e1452e8b26c0b3a52fb65371427d71baeb</x:v>
+        <x:v>feat/0.7.1-candidate @ 37b4195acb5dd9db3cef2bc0ba225af1c368529b | tree 368714246c7f227f63cc1c7548b90eacd6631585</x:v>
       </x:c>
       <x:c r="D6" s="23" t="str">
-        <x:v>feat/protected-content-uiux-reconstruction @ 8e5eb88b8ec566a9ff3261efa84e1fc9a6b1f5c3 | tree 584f59e1452e8b26c0b3a52fb65371427d71baeb</x:v>
+        <x:v>feat/0.7.1-candidate @ 37b4195acb5dd9db3cef2bc0ba225af1c368529b | tree 368714246c7f227f63cc1c7548b90eacd6631585</x:v>
       </x:c>
       <x:c r="E6" s="23" t="str">
-        <x:v>feat/protected-content-uiux-reconstruction @ 8e5eb88b8ec566a9ff3261efa84e1fc9a6b1f5c3 | tree 584f59e1452e8b26c0b3a52fb65371427d71baeb</x:v>
+        <x:v>feat/0.7.1-candidate @ 37b4195acb5dd9db3cef2bc0ba225af1c368529b | tree 368714246c7f227f63cc1c7548b90eacd6631585</x:v>
       </x:c>
       <x:c r="F6" s="23" t="str">
-        <x:v>feat/protected-content-uiux-reconstruction @ 8e5eb88b8ec566a9ff3261efa84e1fc9a6b1f5c3 | tree 584f59e1452e8b26c0b3a52fb65371427d71baeb</x:v>
+        <x:v>feat/0.7.1-candidate @ 37b4195acb5dd9db3cef2bc0ba225af1c368529b | tree 368714246c7f227f63cc1c7548b90eacd6631585</x:v>
       </x:c>
       <x:c r="G6" s="3"/>
       <x:c r="H6" s="3" t="str">
@@ -32605,16 +32605,16 @@
         <x:v>Installed baseline</x:v>
       </x:c>
       <x:c r="C7" s="23" t="str">
-        <x:v>source-home profile: 41 selected components; 33 installed capsule manifests; 22 UI/content/shell capsules. The auditor observed 16 launcher targets through Sky AX; this was not a user-reported list.</x:v>
+        <x:v>Isolated source-home install on localhost:61380: 33 installed capsule manifests and 16 launcher targets. Existing account, passkey, Wallet, and user data remain in the isolated test root.</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
-        <x:v>source-home profile: 41 selected components; 33 installed capsule manifests; 22 UI/content/shell capsules. The auditor observed 16 launcher targets through Sky AX; this was not a user-reported list.</x:v>
+        <x:v>Isolated source-home install on localhost:61380: 33 installed capsule manifests and 16 launcher targets. Existing account, passkey, Wallet, and user data remain in the isolated test root.</x:v>
       </x:c>
       <x:c r="E7" s="23" t="str">
-        <x:v>source-home profile: 41 selected components; 33 installed capsule manifests; 22 UI/content/shell capsules. The auditor observed 16 launcher targets through Sky AX; this was not a user-reported list.</x:v>
+        <x:v>Isolated source-home install on localhost:61380: 33 installed capsule manifests and 16 launcher targets. Existing account, passkey, Wallet, and user data remain in the isolated test root.</x:v>
       </x:c>
       <x:c r="F7" s="23" t="str">
-        <x:v>source-home profile: 41 selected components; 33 installed capsule manifests; 22 UI/content/shell capsules. The auditor observed 16 launcher targets through Sky AX; this was not a user-reported list.</x:v>
+        <x:v>Isolated source-home install on localhost:61380: 33 installed capsule manifests and 16 launcher targets. Existing account, passkey, Wallet, and user data remain in the isolated test root.</x:v>
       </x:c>
       <x:c r="G7" s="3"/>
       <x:c r="H7" s="3" t="str">
@@ -32639,16 +32639,16 @@
         <x:v>Manifest SHA-256</x:v>
       </x:c>
       <x:c r="C8" s="23" t="str">
-        <x:v>8bc5f0a508343b93607cf1fbfef99a3ec291298e4547bdd11304aef246d6d4cf</x:v>
+        <x:v>76eb9ed880aebf6a0e71256c88d38e2966eaee96be34b998475e3ddca2f79dc6</x:v>
       </x:c>
       <x:c r="D8" s="23" t="str">
-        <x:v>8bc5f0a508343b93607cf1fbfef99a3ec291298e4547bdd11304aef246d6d4cf</x:v>
+        <x:v>76eb9ed880aebf6a0e71256c88d38e2966eaee96be34b998475e3ddca2f79dc6</x:v>
       </x:c>
       <x:c r="E8" s="23" t="str">
-        <x:v>8bc5f0a508343b93607cf1fbfef99a3ec291298e4547bdd11304aef246d6d4cf</x:v>
+        <x:v>76eb9ed880aebf6a0e71256c88d38e2966eaee96be34b998475e3ddca2f79dc6</x:v>
       </x:c>
       <x:c r="F8" s="23" t="str">
-        <x:v>8bc5f0a508343b93607cf1fbfef99a3ec291298e4547bdd11304aef246d6d4cf</x:v>
+        <x:v>76eb9ed880aebf6a0e71256c88d38e2966eaee96be34b998475e3ddca2f79dc6</x:v>
       </x:c>
       <x:c r="G8" s="3"/>
       <x:c r="H8" s="3" t="str">
@@ -32707,16 +32707,16 @@
         <x:v>Live tool state</x:v>
       </x:c>
       <x:c r="C10" s="23" t="str">
-        <x:v>Brave reuses the existing signed-in session. All 23 original tabs remain, plus one audit tab. Nested click/fill limitations use verified screenshot clicks and per-key input. Only named audit fixtures are added.</x:v>
+        <x:v>Brave uses the existing signed-in test session. Computer Use reached Home through accessibility controls at 100% zoom. Existing tabs and account data were preserved; tool-control errors remain separate from product results.</x:v>
       </x:c>
       <x:c r="D10" s="23" t="str">
-        <x:v>Brave reuses the existing signed-in session. All 23 original tabs remain, plus one audit tab. Nested click/fill limitations use verified screenshot clicks and per-key input. Only named audit fixtures are added.</x:v>
+        <x:v>Brave uses the existing signed-in test session. Computer Use reached Home through accessibility controls at 100% zoom. Existing tabs and account data were preserved; tool-control errors remain separate from product results.</x:v>
       </x:c>
       <x:c r="E10" s="23" t="str">
-        <x:v>Brave reuses the existing signed-in session. All 23 original tabs remain, plus one audit tab. Nested click/fill limitations use verified screenshot clicks and per-key input. Only named audit fixtures are added.</x:v>
+        <x:v>Brave uses the existing signed-in test session. Computer Use reached Home through accessibility controls at 100% zoom. Existing tabs and account data were preserved; tool-control errors remain separate from product results.</x:v>
       </x:c>
       <x:c r="F10" s="23" t="str">
-        <x:v>Brave reuses the existing signed-in session. All 23 original tabs remain, plus one audit tab. Nested click/fill limitations use verified screenshot clicks and per-key input. Only named audit fixtures are added.</x:v>
+        <x:v>Brave uses the existing signed-in test session. Computer Use reached Home through accessibility controls at 100% zoom. Existing tabs and account data were preserved; tool-control errors remain separate from product results.</x:v>
       </x:c>
       <x:c r="G10" s="3"/>
       <x:c r="H10" s="3" t="str">
@@ -32913,16 +32913,16 @@
         <x:v>Model distinctions</x:v>
       </x:c>
       <x:c r="C17" s="23" t="str">
-        <x:v>F-02 Init is repaired and installed at bd61484c. Zero configured offers is valid; execution needs an approved offer. Remote Profile offers/grants and a compatible weights-CID loader remain separate work.</x:v>
+        <x:v>The installed candidate starts model-provider through the shared Init contract and reaches a truthful zero-offer state. Model execution needs one approved compatible offer. Remote Profile offers and content-addressed model retrieval remain separate journeys.</x:v>
       </x:c>
       <x:c r="D17" s="23" t="str">
-        <x:v>F-02 Init is repaired and installed at bd61484c. Zero configured offers is valid; execution needs an approved offer. Remote Profile offers/grants and a compatible weights-CID loader remain separate work.</x:v>
+        <x:v>The installed candidate starts model-provider through the shared Init contract and reaches a truthful zero-offer state. Model execution needs one approved compatible offer. Remote Profile offers and content-addressed model retrieval remain separate journeys.</x:v>
       </x:c>
       <x:c r="E17" s="23" t="str">
-        <x:v>F-02 Init is repaired and installed at bd61484c. Zero configured offers is valid; execution needs an approved offer. Remote Profile offers/grants and a compatible weights-CID loader remain separate work.</x:v>
+        <x:v>The installed candidate starts model-provider through the shared Init contract and reaches a truthful zero-offer state. Model execution needs one approved compatible offer. Remote Profile offers and content-addressed model retrieval remain separate journeys.</x:v>
       </x:c>
       <x:c r="F17" s="23" t="str">
-        <x:v>F-02 Init is repaired and installed at bd61484c. Zero configured offers is valid; execution needs an approved offer. Remote Profile offers/grants and a compatible weights-CID loader remain separate work.</x:v>
+        <x:v>The installed candidate starts model-provider through the shared Init contract and reaches a truthful zero-offer state. Model execution needs one approved compatible offer. Remote Profile offers and content-addressed model retrieval remain separate journeys.</x:v>
       </x:c>
       <x:c r="G17" s="3"/>
       <x:c r="H17" s="3"/>
@@ -33017,16 +33017,16 @@
         <x:v>Handoff state</x:v>
       </x:c>
       <x:c r="C21" s="23" t="str">
-        <x:v>Installed audit snapshot: b233d832 / tree 3f073277. E-105 binds Runtime, native Home CLI, object-provider and 19 UI assets. Later source changes require separate installed verification.</x:v>
+        <x:v>Installed candidate snapshot: 37b4195a / tree 36871424. Runtime SHA-256 d9c9378b881072c0adc1b534429d7dd87c9cb8240849e677fb8c16c3d1ddc5a8; Home asset SHA-256 7bbffd989be301c9851ee3561bddc4182ec23ced8c502c3f01cdab4f7bb808f7. E-108 records current installed proof.</x:v>
       </x:c>
       <x:c r="D21" s="23" t="str">
-        <x:v>Installed audit snapshot: b233d832 / tree 3f073277. E-105 binds Runtime, native Home CLI, object-provider and 19 UI assets. Later source changes require separate installed verification.</x:v>
+        <x:v>Installed candidate snapshot: 37b4195a / tree 36871424. Runtime SHA-256 d9c9378b881072c0adc1b534429d7dd87c9cb8240849e677fb8c16c3d1ddc5a8; Home asset SHA-256 7bbffd989be301c9851ee3561bddc4182ec23ced8c502c3f01cdab4f7bb808f7. E-108 records current installed proof.</x:v>
       </x:c>
       <x:c r="E21" s="23" t="str">
-        <x:v>Installed audit snapshot: b233d832 / tree 3f073277. E-105 binds Runtime, native Home CLI, object-provider and 19 UI assets. Later source changes require separate installed verification.</x:v>
+        <x:v>Installed candidate snapshot: 37b4195a / tree 36871424. Runtime SHA-256 d9c9378b881072c0adc1b534429d7dd87c9cb8240849e677fb8c16c3d1ddc5a8; Home asset SHA-256 7bbffd989be301c9851ee3561bddc4182ec23ced8c502c3f01cdab4f7bb808f7. E-108 records current installed proof.</x:v>
       </x:c>
       <x:c r="F21" s="23" t="str">
-        <x:v>Installed audit snapshot: b233d832 / tree 3f073277. E-105 binds Runtime, native Home CLI, object-provider and 19 UI assets. Later source changes require separate installed verification.</x:v>
+        <x:v>Installed candidate snapshot: 37b4195a / tree 36871424. Runtime SHA-256 d9c9378b881072c0adc1b534429d7dd87c9cb8240849e677fb8c16c3d1ddc5a8; Home asset SHA-256 7bbffd989be301c9851ee3561bddc4182ec23ced8c502c3f01cdab4f7bb808f7. E-108 records current installed proof.</x:v>
       </x:c>
       <x:c r="G21" s="3"/>
       <x:c r="H21" s="3"/>
@@ -33043,16 +33043,16 @@
         <x:v>Known live evidence</x:v>
       </x:c>
       <x:c r="C22" s="23" t="str">
-        <x:v>61 findings recorded, including the installation metadata gap. Each journey and control retains its result or explicit blocker.</x:v>
+        <x:v>The workbook retains 61 product findings. E-108 adds current installed evidence without changing older outcomes that still need a direct retest.</x:v>
       </x:c>
       <x:c r="D22" s="23" t="str">
-        <x:v>61 findings recorded, including the installation metadata gap. Each journey and control retains its result or explicit blocker.</x:v>
+        <x:v>The workbook retains 61 product findings. E-108 adds current installed evidence without changing older outcomes that still need a direct retest.</x:v>
       </x:c>
       <x:c r="E22" s="23" t="str">
-        <x:v>61 findings recorded, including the installation metadata gap. Each journey and control retains its result or explicit blocker.</x:v>
+        <x:v>The workbook retains 61 product findings. E-108 adds current installed evidence without changing older outcomes that still need a direct retest.</x:v>
       </x:c>
       <x:c r="F22" s="23" t="str">
-        <x:v>61 findings recorded, including the installation metadata gap. Each journey and control retains its result or explicit blocker.</x:v>
+        <x:v>The workbook retains 61 product findings. E-108 adds current installed evidence without changing older outcomes that still need a direct retest.</x:v>
       </x:c>
       <x:c r="G22" s="3"/>
       <x:c r="H22" s="3"/>
@@ -40651,6 +40651,26 @@
       </x:c>
       <x:c r="F332" s="36" t="str">
         <x:v>Original results preserved. New review tab separates 18 retained fixes, 4 verification gates, 32 active issues and 7 setup/scope/release gates. Incoming stage cleanup issue recorded; no live retest or user-state mutation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="333">
+      <x:c r="A333" t="str">
+        <x:v>E-108</x:v>
+      </x:c>
+      <x:c r="B333" t="str">
+        <x:v>Current candidate installed acceptance</x:v>
+      </x:c>
+      <x:c r="C333" t="str">
+        <x:v>Managed provider resolution, launcher coverage, model readiness, Library visibility, and Browser close cleanup</x:v>
+      </x:c>
+      <x:c r="D333" t="str">
+        <x:v>Direct source, installed hashes, Runtime logs, Brave accessibility state, and process inspection</x:v>
+      </x:c>
+      <x:c r="E333" t="str">
+        <x:v>Clean 37b4195a / tree 36871424; localhost:61380; gateway 97275; managed Runtime 97650</x:v>
+      </x:c>
+      <x:c r="F333" t="str">
+        <x:v>Runtime and Home hashes match the isolated install. All 16 launcher targets open. Browser reached Ready in 38.5 seconds and left zero VM, VZ, TURN, or QEMU process residue after Home Close. Existing account and user data were preserved.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -40701,7 +40721,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20fcccf303e34ef8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc35b5f9d21b945a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -43663,7 +43683,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99f391df0aa14d98"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb003a05f3a641cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: close model and owner enrollment source integration
</commit_message>
<xml_diff>
--- a/docs/audits/ElastOS-Home-Journey-Audit.xlsx
+++ b/docs/audits/ElastOS-Home-Journey-Audit.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="1" r:id="R3750605e5f55415a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journey Matrix" sheetId="2" r:id="R41094babc9824b7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Index" sheetId="3" r:id="R2c6710fdd154464c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="4" r:id="R10c8b7c453fb44b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prioritized Plan" sheetId="5" r:id="R6fbcb4f0c7d24123"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me + Evidence" sheetId="6" r:id="R8db7feecbd184105"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Principles Review" sheetId="7" r:id="R92334268b0c04985"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="1" r:id="Rd303ead8adae4b83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journey Matrix" sheetId="2" r:id="R25604c9bb2da4545"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Index" sheetId="3" r:id="Rebc861f5a6f54b3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="4" r:id="R252f8b61e61d4b01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prioritized Plan" sheetId="5" r:id="Rbbda67d1d6704f8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me + Evidence" sheetId="6" r:id="Rdccc12ef3f274e1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Principles Review" sheetId="7" r:id="R43547c75b7dc4fb6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -790,8 +790,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="JourneyMatrix" displayName="JourneyMatrix" ref="A6:U201" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:U201"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="JourneyMatrix" displayName="JourneyMatrix" ref="A6:U204" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:U204"/>
   <x:tableColumns count="21">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Area"/>
@@ -1241,8 +1241,8 @@
         <x:v>Journeys mapped</x:v>
       </x:c>
       <x:c r="C5" s="30" t="n">
-        <x:f>COUNTA('Journey Matrix'!$A$7:$A$201)</x:f>
-        <x:v>195</x:v>
+        <x:f>COUNTA('Journey Matrix'!$A$7:$A$204)</x:f>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="D5" s="29" t="str">
         <x:v>Source inventory, not tests passed.</x:v>
@@ -1385,8 +1385,8 @@
         <x:v>Applicable GUI journeys</x:v>
       </x:c>
       <x:c r="C9" s="30" t="n">
-        <x:f>SUM('Journey Matrix'!$T$7:$T$201)</x:f>
-        <x:v>179</x:v>
+        <x:f>SUM('Journey Matrix'!$T$7:$T$204)</x:f>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="D9" s="29" t="str">
         <x:v>Excludes source-only scope and explicit Not applicable.</x:v>
@@ -1421,7 +1421,7 @@
         <x:v>Observed GUI journeys</x:v>
       </x:c>
       <x:c r="C10" s="30" t="n">
-        <x:f>SUM('Journey Matrix'!$R$7:$R$201)</x:f>
+        <x:f>SUM('Journey Matrix'!$R$7:$R$204)</x:f>
         <x:v>106</x:v>
       </x:c>
       <x:c r="D10" s="29" t="str">
@@ -1457,7 +1457,7 @@
         <x:v>Passed GUI journeys</x:v>
       </x:c>
       <x:c r="C11" s="30" t="n">
-        <x:f>SUM('Journey Matrix'!$S$7:$S$201)</x:f>
+        <x:f>SUM('Journey Matrix'!$S$7:$S$204)</x:f>
         <x:v>19</x:v>
       </x:c>
       <x:c r="D11" s="29" t="str">
@@ -1494,7 +1494,7 @@
       </x:c>
       <x:c r="C12" s="31" t="n">
         <x:f>IFERROR(C10/C9,0)</x:f>
-        <x:v>0.5921787709497207</x:v>
+        <x:v>0.5824175824175825</x:v>
       </x:c>
       <x:c r="D12" s="29" t="str">
         <x:v>Observed / applicable GUI journeys. Partial observations remain incomplete.</x:v>
@@ -1637,7 +1637,7 @@
         <x:v>Tool-blocked journeys</x:v>
       </x:c>
       <x:c r="C16" s="30" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D16" s="29" t="str">
@@ -1673,8 +1673,8 @@
         <x:v>Live prerequisite blockers</x:v>
       </x:c>
       <x:c r="C17" s="30" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
-        <x:v>76</x:v>
+        <x:f>COUNTIF('Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="D17" s="29" t="str">
         <x:v>Configuration/fixtures needed before controlled execution.</x:v>
@@ -1781,7 +1781,7 @@
         <x:v>Full journeys completed</x:v>
       </x:c>
       <x:c r="C20" s="30" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$Q$7:$Q$201,'Read Me + Evidence'!$K$11,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$7)+COUNTIFS('Journey Matrix'!$Q$7:$Q$201,'Read Me + Evidence'!$K$11,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$Q$7:$Q$204,'Read Me + Evidence'!$K$11,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$7)+COUNTIFS('Journey Matrix'!$Q$7:$Q$204,'Read Me + Evidence'!$K$11,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>54</x:v>
       </x:c>
       <x:c r="D20" s="29" t="str">
@@ -1818,7 +1818,7 @@
       </x:c>
       <x:c r="C21" s="31" t="n">
         <x:f>IFERROR(C20/C9,0)</x:f>
-        <x:v>0.3016759776536313</x:v>
+        <x:v>0.2967032967032967</x:v>
       </x:c>
       <x:c r="D21" s="29" t="str">
         <x:v>Full completed journeys / applicable GUI journeys. Source mapping is a different measure.</x:v>
@@ -1981,35 +1981,35 @@
         <x:v>archive-manager</x:v>
       </x:c>
       <x:c r="B27" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A27)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A27)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="C27" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A27)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A27)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D27" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A27)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A27)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E27" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A27)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A27)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F27" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A27,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A27,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="G27" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A27,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A27,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="H27" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A27,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A27,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I27" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A27,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A27,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="J27" s="3" t="str">
@@ -2025,35 +2025,35 @@
         <x:v>assistant</x:v>
       </x:c>
       <x:c r="B28" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A28)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A28)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="C28" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A28)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A28)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="D28" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A28)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A28)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E28" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A28)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A28)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="F28" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A28,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A28,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G28" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A28,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A28,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="H28" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A28,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A28,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I28" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A28,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A28,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="J28" s="3" t="str">
@@ -2069,35 +2069,35 @@
         <x:v>browser</x:v>
       </x:c>
       <x:c r="B29" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A29)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A29)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="C29" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A29)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A29)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="D29" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A29)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A29)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="E29" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A29)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A29)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F29" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A29,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A29,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="G29" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A29,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A29,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="H29" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A29,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A29,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="I29" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A29,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A29,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="J29" s="3" t="str">
@@ -2113,35 +2113,35 @@
         <x:v>chat-room</x:v>
       </x:c>
       <x:c r="B30" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A30)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A30)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="C30" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A30)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A30)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D30" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A30)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A30)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="E30" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A30)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A30)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="F30" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A30,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A30,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="G30" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A30,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A30,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="H30" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A30,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A30,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I30" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A30,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A30,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="J30" s="3" t="str">
@@ -2157,35 +2157,35 @@
         <x:v>documents</x:v>
       </x:c>
       <x:c r="B31" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A31)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A31)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="C31" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A31)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A31)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="D31" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A31)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A31)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E31" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A31)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A31)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="F31" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A31,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A31,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="G31" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A31,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A31,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="H31" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A31,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A31,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I31" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A31,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A31,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="J31" s="3" t="str">
@@ -2201,35 +2201,35 @@
         <x:v>elacity-player</x:v>
       </x:c>
       <x:c r="B32" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A32)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A32)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C32" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A32)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A32)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D32" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A32)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A32)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E32" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A32)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A32)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F32" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A32,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A32,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G32" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A32,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A32,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H32" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A32,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A32,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I32" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A32,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A32,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="J32" s="3" t="str">
@@ -2245,35 +2245,35 @@
         <x:v>gba-emulator</x:v>
       </x:c>
       <x:c r="B33" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A33)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A33)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C33" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A33)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A33)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D33" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A33)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A33)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E33" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A33)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A33)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F33" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A33,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A33,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="G33" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A33,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A33,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="H33" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A33,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A33,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I33" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A33,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A33,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J33" s="3" t="str">
@@ -2289,35 +2289,35 @@
         <x:v>gba-nonogram</x:v>
       </x:c>
       <x:c r="B34" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A34)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A34)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C34" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A34)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A34)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D34" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A34)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A34)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E34" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A34)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A34)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F34" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A34,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A34,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G34" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A34,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A34,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H34" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A34,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A34,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I34" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A34,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A34,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J34" s="3" t="str">
@@ -2333,35 +2333,35 @@
         <x:v>gba-ucity</x:v>
       </x:c>
       <x:c r="B35" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A35)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A35)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C35" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A35)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A35)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D35" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A35)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A35)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E35" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A35)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A35)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F35" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A35,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A35,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="G35" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A35,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A35,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H35" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A35,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A35,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I35" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A35,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A35,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J35" s="3" t="str">
@@ -2377,36 +2377,36 @@
         <x:v>home</x:v>
       </x:c>
       <x:c r="B36" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A36)</x:f>
-        <x:v>7</x:v>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A36)</x:f>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C36" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A36)</x:f>
-        <x:v>7</x:v>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A36)</x:f>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D36" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A36)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A36)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E36" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A36)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A36)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F36" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A36,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A36,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G36" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A36,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A36,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H36" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A36,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A36,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I36" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A36,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
-        <x:v>6</x:v>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A36,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="J36" s="3" t="str">
         <x:v>Yes</x:v>
@@ -2421,35 +2421,35 @@
         <x:v>home-cli</x:v>
       </x:c>
       <x:c r="B37" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A37)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A37)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C37" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A37)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A37)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D37" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A37)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A37)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="E37" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A37)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A37)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F37" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A37,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A37,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="G37" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A37,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A37,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H37" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A37,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A37,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I37" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A37,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A37,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="J37" s="3" t="str">
@@ -2465,35 +2465,35 @@
         <x:v>home-gui</x:v>
       </x:c>
       <x:c r="B38" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A38)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A38)</x:f>
         <x:v>16</x:v>
       </x:c>
       <x:c r="C38" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A38)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A38)</x:f>
         <x:v>16</x:v>
       </x:c>
       <x:c r="D38" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A38)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A38)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="E38" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A38)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A38)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="F38" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A38,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A38,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="G38" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A38,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A38,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="H38" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A38,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A38,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I38" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A38,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A38,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="J38" s="3" t="str">
@@ -2509,35 +2509,35 @@
         <x:v>inbox</x:v>
       </x:c>
       <x:c r="B39" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A39)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A39)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="C39" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A39)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A39)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="D39" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A39)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A39)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="E39" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A39)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A39)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F39" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A39,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A39,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G39" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A39,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A39,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="H39" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A39,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A39,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I39" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A39,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A39,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="J39" s="3" t="str">
@@ -2553,35 +2553,35 @@
         <x:v>library</x:v>
       </x:c>
       <x:c r="B40" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A40)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A40)</x:f>
         <x:v>24</x:v>
       </x:c>
       <x:c r="C40" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A40)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A40)</x:f>
         <x:v>23</x:v>
       </x:c>
       <x:c r="D40" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A40)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A40)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="E40" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A40)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A40)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="F40" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A40,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A40,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="G40" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A40,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A40,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="H40" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A40,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A40,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I40" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A40,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A40,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="J40" s="3" t="str">
@@ -2597,35 +2597,35 @@
         <x:v>marketplace</x:v>
       </x:c>
       <x:c r="B41" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A41)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A41)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="C41" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A41)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A41)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D41" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A41)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A41)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E41" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A41)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A41)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="F41" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A41,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A41,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="G41" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A41,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A41,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="H41" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A41,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A41,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I41" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A41,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A41,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="J41" s="3" t="str">
@@ -2641,35 +2641,35 @@
         <x:v>people</x:v>
       </x:c>
       <x:c r="B42" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A42)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A42)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="C42" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A42)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A42)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D42" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A42)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A42)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="E42" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A42)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A42)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F42" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A42,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A42,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G42" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A42,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A42,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="H42" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A42,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A42,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I42" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A42,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A42,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="J42" s="3" t="str">
@@ -2685,35 +2685,35 @@
         <x:v>services</x:v>
       </x:c>
       <x:c r="B43" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A43)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A43)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="C43" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A43)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A43)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D43" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A43)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A43)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="E43" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A43)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A43)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F43" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A43,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A43,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G43" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A43,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A43,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="H43" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A43,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A43,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I43" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A43,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A43,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="J43" s="3" t="str">
@@ -2729,35 +2729,35 @@
         <x:v>system</x:v>
       </x:c>
       <x:c r="B44" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A44)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A44)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="C44" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A44)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A44)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="D44" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A44)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A44)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E44" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A44)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A44)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="F44" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A44,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A44,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="G44" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A44,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A44,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="H44" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A44,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A44,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I44" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A44,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A44,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="J44" s="3" t="str">
@@ -2773,35 +2773,35 @@
         <x:v>wallet</x:v>
       </x:c>
       <x:c r="B45" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A45)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A45)</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="C45" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A45)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A45)</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="D45" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A45)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A45)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="E45" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A45)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A45)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F45" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A45,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A45,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G45" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A45,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A45,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="H45" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A45,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A45,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I45" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A45,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A45,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="J45" s="3" t="str">
@@ -2817,35 +2817,35 @@
         <x:v>wallet-metamask</x:v>
       </x:c>
       <x:c r="B46" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A46)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A46)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C46" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A46)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A46)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D46" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A46)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A46)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E46" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A46)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A46)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F46" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A46,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A46,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G46" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A46,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A46,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H46" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A46,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A46,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I46" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A46,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A46,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="J46" s="3" t="str">
@@ -2861,35 +2861,35 @@
         <x:v>wallet-unisat</x:v>
       </x:c>
       <x:c r="B47" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A47)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A47)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C47" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A47)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A47)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D47" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A47)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A47)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E47" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A47)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A47)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F47" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A47,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A47,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G47" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A47,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A47,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H47" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A47,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A47,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I47" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A47,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A47,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="J47" s="3" t="str">
@@ -2905,35 +2905,35 @@
         <x:v>wallet-walletconnect</x:v>
       </x:c>
       <x:c r="B48" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A48)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A48)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C48" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A48)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A48)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D48" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A48)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A48)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E48" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A48)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A48)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F48" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A48,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A48,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G48" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A48,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A48,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H48" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A48,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A48,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I48" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A48,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A48,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="J48" s="3" t="str">
@@ -2949,35 +2949,35 @@
         <x:v>model-provider</x:v>
       </x:c>
       <x:c r="B49" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A49)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A49)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="C49" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A49)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A49)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D49" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A49)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A49)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E49" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A49)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A49)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F49" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A49,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A49,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G49" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A49,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A49,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H49" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A49,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A49,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I49" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A49,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A49,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="J49" s="3" t="str">
@@ -2993,35 +2993,35 @@
         <x:v>runtime-services</x:v>
       </x:c>
       <x:c r="B50" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A50)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A50)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="C50" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A50)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A50)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D50" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A50)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A50)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E50" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A50)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A50)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F50" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A50,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A50,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="G50" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A50,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A50,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="H50" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A50,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A50,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I50" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A50,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A50,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="J50" s="3" t="str">
@@ -3037,35 +3037,35 @@
         <x:v>shared</x:v>
       </x:c>
       <x:c r="B51" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A51)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A51)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C51" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A51)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A51)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D51" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A51)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A51)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="E51" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A51)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A51)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F51" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A51,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A51,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="G51" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A51,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A51,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H51" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A51,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A51,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I51" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A51,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A51,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J51" s="3" t="str">
@@ -3131,7 +3131,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50c9a5ba1c38444f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cf337f3dcdb4cf4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3444,7 +3444,9 @@
         <x:f>IF(AND(Q7='Read Me + Evidence'!$K$11,D7&lt;&gt;'Read Me + Evidence'!$H$12),1,0)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="U7" s="3" t="str"/>
+      <x:c r="U7" s="3" t="str">
+        <x:v>Source 145fec2b, eb25f747, 43b8f830: exact RP/origin ceremony; secure credential persistence; one durable owner operation. Gateway 60, direct handlers 10, owner 7 and identity 48 tests pass. Installed first-owner proof remains open.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="153" customHeight="1">
       <x:c r="A8" s="3" t="str">
@@ -3509,7 +3511,9 @@
         <x:f>IF(AND(Q8='Read Me + Evidence'!$K$11,D8&lt;&gt;'Read Me + Evidence'!$H$12),1,0)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="U8" s="3" t="str"/>
+      <x:c r="U8" s="3" t="str">
+        <x:v>Source 43b8f830: sign-in resolves an existing active proof binding; orphan credentials cannot create authority. Expired terminal enrollment grants require normal sign-in. Installed verdict unchanged.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="153" customHeight="1">
       <x:c r="A9" s="3" t="str">
@@ -3573,7 +3577,9 @@
         <x:f>IF(AND(Q9='Read Me + Evidence'!$K$11,D9&lt;&gt;'Read Me + Evidence'!$H$12),1,0)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="U9" s="3" t="str"/>
+      <x:c r="U9" s="3" t="str">
+        <x:v>Source 43b8f830: both registration routes require enabled guest policy and a live Admin before credential effects. Revocation after begin is denied with unchanged stored credentials. Installed policy proof remains open.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="153" customHeight="1">
       <x:c r="A10" s="3" t="str">
@@ -3766,7 +3772,9 @@
         <x:f>IF(AND(Q12='Read Me + Evidence'!$K$11,D12&lt;&gt;'Read Me + Evidence'!$H$12),1,0)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="U12" s="3" t="str"/>
+      <x:c r="U12" s="3" t="str">
+        <x:v>Source 43b8f830: typed 403 denials; exact claimant recovery after response loss; expiry, revoked binding, concurrent claimant and restart fixtures pass. Installed cancellation/recovery proof remains open.</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="153" customHeight="1">
       <x:c r="A13" s="3" t="str">
@@ -13589,7 +13597,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="U163" s="3" t="str">
-        <x:v>The provider lifecycle is installed and healthy. Model execution begins after an operator selects and configures an approved offer.</x:v>
+        <x:v>Source c95cf4c9 and 7c4fc929: verified bootstrap artifacts and bounded local engine lifecycle. Combined model provider tests pass (182 unit, 5 process; one existing ignored case). Existing installed verdict is unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="164" ht="153" customHeight="1">
@@ -13656,7 +13664,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="U164" s="3" t="str">
-        <x:v>First-model selection/download UX is proposed and needs a decision. source-home installs model-provider but selects neither weights nor a model backend; this end-user flow is not built or tested.</x:v>
+        <x:v>Source c95cf4c9/7c4fc929 verifies local engine/model bytes and child lifecycle; fcb8fc5e/0d768415 has hosted/Responses fixtures. Home Agent Stop can persist Stopped before Runtime settles failed/unknown cancellation. UI proof must retain providerRunId and reconcile Runtime state. CID Get remains planned in ed275ba0. Installed first-offer and cancellation proof remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="165" ht="153" customHeight="1">
@@ -13723,7 +13731,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="U165" s="3" t="str">
-        <x:v>Missing configuration is a valid zero-offer state. Invalid configuration remains a separate failure branch; useful setup guidance still needs live review.</x:v>
+        <x:v>Combined source model tests preserve missing-config zero offers and invalid-config refusal. Hosted terminal evidence and honest unknown cancellation settlement have fixture coverage; installed negative configuration proof remains open.</x:v>
       </x:c>
     </x:row>
     <x:row r="166" ht="153" customHeight="1">
@@ -16081,6 +16089,200 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="U201" s="3" t="str"/>
+    </x:row>
+    <x:row r="202" ht="220" customHeight="1">
+      <x:c r="A202" s="36" t="str">
+        <x:v>AUTH-08</x:v>
+      </x:c>
+      <x:c r="B202" s="36" t="str">
+        <x:v>Home / sign-in</x:v>
+      </x:c>
+      <x:c r="C202" s="36" t="str">
+        <x:v>Operator-admitted HTTPS first owner</x:v>
+      </x:c>
+      <x:c r="D202" s="36" t="str">
+        <x:v>Blocked prerequisite</x:v>
+      </x:c>
+      <x:c r="E202" s="36" t="str">
+        <x:v>Runtime admits one first owner after operator authorization bound to the exact HTTPS origin and RP, followed by user passkey consent.</x:v>
+      </x:c>
+      <x:c r="F202" s="36" t="str">
+        <x:v>Source fixtures only; installed public-origin enrollment remains open.</x:v>
+      </x:c>
+      <x:c r="G202" s="36" t="str">
+        <x:v>controlled-identity</x:v>
+      </x:c>
+      <x:c r="H202" s="36" t="str">
+        <x:v>implemented-source</x:v>
+      </x:c>
+      <x:c r="I202" s="36" t="str">
+        <x:v>Operator enrollment token; Name; Use passkey</x:v>
+      </x:c>
+      <x:c r="J202" s="36" t="str">
+        <x:v>1. Arm one disposable HTTPS Home
+2. Enroll with the approved token and a user-operated passkey
+3. Confirm one Admin account</x:v>
+      </x:c>
+      <x:c r="K202" s="36" t="str">
+        <x:v>Fresh disposable Home; supported secure host; explicit operator and user consent</x:v>
+      </x:c>
+      <x:c r="L202" s="36"/>
+      <x:c r="M202" s="36"/>
+      <x:c r="N202" s="36"/>
+      <x:c r="O202" s="36" t="str">
+        <x:v>43b8f830; elastos/crates/elastos-server/src/auth.rs; api/auth_gateway.rs; api/handlers/identity.rs; scripts/home-owner-enrollment-smoke.mjs</x:v>
+      </x:c>
+      <x:c r="P202" s="36" t="str">
+        <x:v>home</x:v>
+      </x:c>
+      <x:c r="Q202" s="36" t="str">
+        <x:v>GUI</x:v>
+      </x:c>
+      <x:c r="R202" s="36" t="n">
+        <x:f>IF(AND(Q202='Read Me + Evidence'!$K$11,OR(D202='Read Me + Evidence'!$H$202,D202='Read Me + Evidence'!$H$8,D202='Read Me + Evidence'!$H$9)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S202" s="36" t="n">
+        <x:f>IF(AND(Q202='Read Me + Evidence'!$K$11,D202='Read Me + Evidence'!$H$202),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T202" s="36" t="n">
+        <x:f>IF(AND(Q202='Read Me + Evidence'!$K$11,D202&lt;&gt;'Read Me + Evidence'!$H$12),1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U202" s="36" t="str">
+        <x:v>Both actual route families pass exact binding, denial and concurrent-owner fixtures. Existing user accounts remain outside this test scope.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="203" ht="220" customHeight="1">
+      <x:c r="A203" s="36" t="str">
+        <x:v>AUTH-09</x:v>
+      </x:c>
+      <x:c r="B203" s="36" t="str">
+        <x:v>Home / sign-in</x:v>
+      </x:c>
+      <x:c r="C203" s="36" t="str">
+        <x:v>Reload after owner completion response loss</x:v>
+      </x:c>
+      <x:c r="D203" s="36" t="str">
+        <x:v>Blocked prerequisite</x:v>
+      </x:c>
+      <x:c r="E203" s="36" t="str">
+        <x:v>The original claimant resumes the same verified owner operation after reload, with the saved name and one terminal grant.</x:v>
+      </x:c>
+      <x:c r="F203" s="36" t="str">
+        <x:v>Source controller and persisted-route fixtures only; installed reload proof remains open.</x:v>
+      </x:c>
+      <x:c r="G203" s="36" t="str">
+        <x:v>controlled-identity</x:v>
+      </x:c>
+      <x:c r="H203" s="36" t="str">
+        <x:v>implemented-source</x:v>
+      </x:c>
+      <x:c r="I203" s="36" t="str">
+        <x:v>Resume Home setup; claimant cookie</x:v>
+      </x:c>
+      <x:c r="J203" s="36" t="str">
+        <x:v>1. Verify a disposable enrollment
+2. Lose its completion response
+3. Reload and resume
+4. Confirm one account, name and grant</x:v>
+      </x:c>
+      <x:c r="K203" s="36" t="str">
+        <x:v>Disposable authorized enrollment; controlled response interruption</x:v>
+      </x:c>
+      <x:c r="L203" s="36"/>
+      <x:c r="M203" s="36"/>
+      <x:c r="N203" s="36"/>
+      <x:c r="O203" s="36" t="str">
+        <x:v>43b8f830; elastos/crates/elastos-server/src/auth.rs; api/auth_gateway.rs; api/handlers/identity.rs; scripts/home-owner-enrollment-smoke.mjs</x:v>
+      </x:c>
+      <x:c r="P203" s="36" t="str">
+        <x:v>home</x:v>
+      </x:c>
+      <x:c r="Q203" s="36" t="str">
+        <x:v>GUI</x:v>
+      </x:c>
+      <x:c r="R203" s="36" t="n">
+        <x:f>IF(AND(Q203='Read Me + Evidence'!$K$11,OR(D203='Read Me + Evidence'!$H$203,D203='Read Me + Evidence'!$H$8,D203='Read Me + Evidence'!$H$9)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S203" s="36" t="n">
+        <x:f>IF(AND(Q203='Read Me + Evidence'!$K$11,D203='Read Me + Evidence'!$H$203),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T203" s="36" t="n">
+        <x:f>IF(AND(Q203='Read Me + Evidence'!$K$11,D203&lt;&gt;'Read Me + Evidence'!$H$12),1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U203" s="36" t="str">
+        <x:v>Home reload smoke and four persistence-boundary restart fixtures pass. Resume needs no second attestation; an expired terminal grant uses normal sign-in.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204" ht="220" customHeight="1">
+      <x:c r="A204" s="36" t="str">
+        <x:v>AUTH-10</x:v>
+      </x:c>
+      <x:c r="B204" s="36" t="str">
+        <x:v>Home / sign-in</x:v>
+      </x:c>
+      <x:c r="C204" s="36" t="str">
+        <x:v>Denied and competing owner enrollment</x:v>
+      </x:c>
+      <x:c r="D204" s="36" t="str">
+        <x:v>Blocked prerequisite</x:v>
+      </x:c>
+      <x:c r="E204" s="36" t="str">
+        <x:v>Wrong claimant, origin, RP, expiry or revoked proof fails closed; concurrent attempts establish at most one owner.</x:v>
+      </x:c>
+      <x:c r="F204" s="36" t="str">
+        <x:v>Source negative fixtures only; installed controlled-denial proof remains open.</x:v>
+      </x:c>
+      <x:c r="G204" s="36" t="str">
+        <x:v>controlled-identity</x:v>
+      </x:c>
+      <x:c r="H204" s="36" t="str">
+        <x:v>implemented-source</x:v>
+      </x:c>
+      <x:c r="I204" s="36" t="str">
+        <x:v>Enrollment refusal; retry</x:v>
+      </x:c>
+      <x:c r="J204" s="36" t="str">
+        <x:v>1. Use invalid or expired disposable admission
+2. Try competing claimants
+3. Restart at persistence boundaries
+4. Confirm exact state and one winner</x:v>
+      </x:c>
+      <x:c r="K204" s="36" t="str">
+        <x:v>Fresh disposable Home; controlled failures; preserve all existing accounts</x:v>
+      </x:c>
+      <x:c r="L204" s="36"/>
+      <x:c r="M204" s="36"/>
+      <x:c r="N204" s="36"/>
+      <x:c r="O204" s="36" t="str">
+        <x:v>43b8f830; elastos/crates/elastos-server/src/auth.rs; api/auth_gateway.rs; api/handlers/identity.rs; scripts/home-owner-enrollment-smoke.mjs</x:v>
+      </x:c>
+      <x:c r="P204" s="36" t="str">
+        <x:v>home</x:v>
+      </x:c>
+      <x:c r="Q204" s="36" t="str">
+        <x:v>GUI</x:v>
+      </x:c>
+      <x:c r="R204" s="36" t="n">
+        <x:f>IF(AND(Q204='Read Me + Evidence'!$K$11,OR(D204='Read Me + Evidence'!$H$204,D204='Read Me + Evidence'!$H$8,D204='Read Me + Evidence'!$H$9)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S204" s="36" t="n">
+        <x:f>IF(AND(Q204='Read Me + Evidence'!$K$11,D204='Read Me + Evidence'!$H$204),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T204" s="36" t="n">
+        <x:f>IF(AND(Q204='Read Me + Evidence'!$K$11,D204&lt;&gt;'Read Me + Evidence'!$H$12),1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U204" s="36" t="str">
+        <x:v>Typed 403 and no-effect route tests pass; concurrent claim/completion and credential-counter/revocation recovery preserve exact ownership.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -16107,14 +16309,17 @@
       <x:formula>"Not run"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="D7:D201">
+      <x:formula1>"Not run,Pass,Fail,Partially observed,Blocked prerequisite,Blocked tool,Not applicable"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D202:D204">
       <x:formula1>"Not run,Pass,Fail,Partially observed,Blocked prerequisite,Blocked tool,Not applicable"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R562c5740ef324d73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd865d76e59b475f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27775,8 +27980,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7017081ee9e147bb"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d7f30e34d784a20"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b679907aa1449cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cd76a6c559e4ca3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30287,7 +30492,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d6ceee7dd914057"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd547cfe09454ea0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32414,7 +32619,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14d89847794342f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc292c811d2b14791"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40721,7 +40926,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc35b5f9d21b945a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re601c2bd9c3344a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -43683,7 +43888,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb003a05f3a641cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R485b724059314d7e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(home): add storefront and canonical Home entry
Serve Home at /home/ with old bookmark redirects, shared capsule policy and stable installed-app identity. Add a responsive storefront that distinguishes hosted source from public installer metadata and keeps unsupported install actions unavailable.

Verified: 31 focused Rust cases, 4 manifest follow-up cases, Home recovery/sign-out smoke, 20 website tests, 6 website checks, entropy and format gates. Desktop/mobile metadata and keyboard checks passed. Seed installation and human target acceptance remain open.
</commit_message>
<xml_diff>
--- a/docs/audits/ElastOS-Home-Journey-Audit.xlsx
+++ b/docs/audits/ElastOS-Home-Journey-Audit.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="1" r:id="R3750605e5f55415a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journey Matrix" sheetId="2" r:id="R41094babc9824b7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Index" sheetId="3" r:id="R2c6710fdd154464c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="4" r:id="R10c8b7c453fb44b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prioritized Plan" sheetId="5" r:id="R6fbcb4f0c7d24123"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me + Evidence" sheetId="6" r:id="R8db7feecbd184105"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Principles Review" sheetId="7" r:id="R92334268b0c04985"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="1" r:id="R91e8907e4cab47a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journey Matrix" sheetId="2" r:id="Rf04a8686ad4c4448"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Index" sheetId="3" r:id="R4ed5471b78d34685"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="4" r:id="R50034081886f4038"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prioritized Plan" sheetId="5" r:id="Rf59f7f48194d4eca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me + Evidence" sheetId="6" r:id="R8f30d66bb1384936"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Principles Review" sheetId="7" r:id="Rb4601da5e97e4ce6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -138,7 +138,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -195,6 +195,11 @@
         <x:fgColor rgb="FFFFF4DC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F8FE"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -202,7 +207,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="58">
+  <x:cellXfs count="59">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -371,11 +376,14 @@
     <x:xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="37">
+  <x:dxfs count="43">
     <x:dxf>
       <x:font>
         <x:color rgb="FF256545"/>
@@ -765,13 +773,73 @@
         </x:patternFill>
       </x:fill>
     </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF256545"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE8F4EC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FFA4262C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCEBED"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF865A12"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF3D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF865A12"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF3D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF65477E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF0EAF7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF55666A"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF3F5F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
   </x:dxfs>
 </x:styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="CoverageByCapsule" displayName="CoverageByCapsule" ref="A26:K51" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A26:K51"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="CoverageByCapsule" displayName="CoverageByCapsule" ref="A26:K52" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A26:K52"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Capsule / area"/>
     <x:tableColumn id="2" name="Mapped"/>
@@ -790,8 +858,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="JourneyMatrix" displayName="JourneyMatrix" ref="A6:U201" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:U201"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="JourneyMatrix" displayName="JourneyMatrix" ref="A6:U204" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:U204"/>
   <x:tableColumns count="21">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Area"/>
@@ -1241,8 +1309,8 @@
         <x:v>Journeys mapped</x:v>
       </x:c>
       <x:c r="C5" s="30" t="n">
-        <x:f>COUNTA('Journey Matrix'!$A$7:$A$201)</x:f>
-        <x:v>195</x:v>
+        <x:f>COUNTA('Journey Matrix'!$A$7:$A$204)</x:f>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="D5" s="29" t="str">
         <x:v>Source inventory, not tests passed.</x:v>
@@ -1313,7 +1381,7 @@
         <x:v>Installed UI capsules mapped</x:v>
       </x:c>
       <x:c r="C7" s="30" t="n">
-        <x:f>COUNTIFS(J27:J51,"Yes",B27:B51,"&gt;0")</x:f>
+        <x:f>COUNTIFS(J27:J52,"Yes",B27:B52,"&gt;0")</x:f>
         <x:v>22</x:v>
       </x:c>
       <x:c r="D7" s="29" t="str">
@@ -1349,7 +1417,7 @@
         <x:v>Source mapping coverage</x:v>
       </x:c>
       <x:c r="C8" s="31" t="n">
-        <x:f>IFERROR(C7/COUNTIF(J27:J51,"Yes"),0)</x:f>
+        <x:f>IFERROR(C7/COUNTIF(J27:J52,"Yes"),0)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D8" s="29" t="str">
@@ -1385,8 +1453,8 @@
         <x:v>Applicable GUI journeys</x:v>
       </x:c>
       <x:c r="C9" s="30" t="n">
-        <x:f>SUM('Journey Matrix'!$T$7:$T$201)</x:f>
-        <x:v>179</x:v>
+        <x:f>SUM('Journey Matrix'!$T$7:$T$204)</x:f>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="D9" s="29" t="str">
         <x:v>Excludes source-only scope and explicit Not applicable.</x:v>
@@ -1421,7 +1489,7 @@
         <x:v>Observed GUI journeys</x:v>
       </x:c>
       <x:c r="C10" s="30" t="n">
-        <x:f>SUM('Journey Matrix'!$R$7:$R$201)</x:f>
+        <x:f>SUM('Journey Matrix'!$R$7:$R$204)</x:f>
         <x:v>106</x:v>
       </x:c>
       <x:c r="D10" s="29" t="str">
@@ -1457,7 +1525,7 @@
         <x:v>Passed GUI journeys</x:v>
       </x:c>
       <x:c r="C11" s="30" t="n">
-        <x:f>SUM('Journey Matrix'!$S$7:$S$201)</x:f>
+        <x:f>SUM('Journey Matrix'!$S$7:$S$204)</x:f>
         <x:v>19</x:v>
       </x:c>
       <x:c r="D11" s="29" t="str">
@@ -1494,7 +1562,7 @@
       </x:c>
       <x:c r="C12" s="31" t="n">
         <x:f>IFERROR(C10/C9,0)</x:f>
-        <x:v>0.5921787709497207</x:v>
+        <x:v>0.5824175824175825</x:v>
       </x:c>
       <x:c r="D12" s="29" t="str">
         <x:v>Observed / applicable GUI journeys. Partial observations remain incomplete.</x:v>
@@ -1637,7 +1705,7 @@
         <x:v>Tool-blocked journeys</x:v>
       </x:c>
       <x:c r="C16" s="30" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D16" s="29" t="str">
@@ -1673,7 +1741,7 @@
         <x:v>Live prerequisite blockers</x:v>
       </x:c>
       <x:c r="C17" s="30" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>76</x:v>
       </x:c>
       <x:c r="D17" s="29" t="str">
@@ -1781,7 +1849,7 @@
         <x:v>Full journeys completed</x:v>
       </x:c>
       <x:c r="C20" s="30" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$Q$7:$Q$201,'Read Me + Evidence'!$K$11,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$7)+COUNTIFS('Journey Matrix'!$Q$7:$Q$201,'Read Me + Evidence'!$K$11,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$Q$7:$Q$204,'Read Me + Evidence'!$K$11,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$7)+COUNTIFS('Journey Matrix'!$Q$7:$Q$204,'Read Me + Evidence'!$K$11,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>54</x:v>
       </x:c>
       <x:c r="D20" s="29" t="str">
@@ -1818,7 +1886,7 @@
       </x:c>
       <x:c r="C21" s="31" t="n">
         <x:f>IFERROR(C20/C9,0)</x:f>
-        <x:v>0.3016759776536313</x:v>
+        <x:v>0.2967032967032967</x:v>
       </x:c>
       <x:c r="D21" s="29" t="str">
         <x:v>Full completed journeys / applicable GUI journeys. Source mapping is a different measure.</x:v>
@@ -1981,35 +2049,35 @@
         <x:v>archive-manager</x:v>
       </x:c>
       <x:c r="B27" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A27)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A27)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="C27" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A27)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A27)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D27" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A27)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A27)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E27" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A27)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A27)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F27" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A27,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A27,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="G27" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A27,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A27,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="H27" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A27,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A27,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I27" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A27,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A27,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="J27" s="3" t="str">
@@ -2025,35 +2093,35 @@
         <x:v>assistant</x:v>
       </x:c>
       <x:c r="B28" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A28)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A28)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="C28" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A28)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A28)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="D28" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A28)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A28)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E28" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A28)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A28)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="F28" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A28,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A28,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G28" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A28,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A28,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="H28" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A28,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A28,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I28" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A28,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A28,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="J28" s="3" t="str">
@@ -2069,35 +2137,35 @@
         <x:v>browser</x:v>
       </x:c>
       <x:c r="B29" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A29)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A29)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="C29" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A29)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A29)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="D29" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A29)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A29)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="E29" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A29)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A29)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F29" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A29,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A29,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="G29" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A29,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A29,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="H29" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A29,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A29,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="I29" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A29,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A29,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="J29" s="3" t="str">
@@ -2113,35 +2181,35 @@
         <x:v>chat-room</x:v>
       </x:c>
       <x:c r="B30" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A30)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A30)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="C30" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A30)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A30)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D30" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A30)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A30)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="E30" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A30)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A30)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="F30" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A30,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A30,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="G30" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A30,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A30,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="H30" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A30,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A30,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I30" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A30,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A30,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="J30" s="3" t="str">
@@ -2157,35 +2225,35 @@
         <x:v>documents</x:v>
       </x:c>
       <x:c r="B31" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A31)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A31)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="C31" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A31)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A31)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="D31" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A31)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A31)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E31" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A31)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A31)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="F31" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A31,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A31,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="G31" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A31,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A31,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="H31" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A31,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A31,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I31" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A31,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A31,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="J31" s="3" t="str">
@@ -2201,35 +2269,35 @@
         <x:v>elacity-player</x:v>
       </x:c>
       <x:c r="B32" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A32)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A32)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C32" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A32)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A32)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D32" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A32)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A32)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E32" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A32)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A32)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F32" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A32,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A32,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G32" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A32,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A32,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H32" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A32,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A32,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I32" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A32,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A32,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="J32" s="3" t="str">
@@ -2245,35 +2313,35 @@
         <x:v>gba-emulator</x:v>
       </x:c>
       <x:c r="B33" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A33)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A33)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C33" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A33)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A33)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D33" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A33)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A33)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E33" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A33)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A33)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F33" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A33,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A33,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="G33" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A33,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A33,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="H33" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A33,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A33,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I33" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A33,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A33,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J33" s="3" t="str">
@@ -2289,35 +2357,35 @@
         <x:v>gba-nonogram</x:v>
       </x:c>
       <x:c r="B34" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A34)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A34)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C34" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A34)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A34)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D34" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A34)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A34)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E34" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A34)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A34)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F34" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A34,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A34,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G34" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A34,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A34,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H34" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A34,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A34,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I34" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A34,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A34,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J34" s="3" t="str">
@@ -2333,35 +2401,35 @@
         <x:v>gba-ucity</x:v>
       </x:c>
       <x:c r="B35" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A35)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A35)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C35" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A35)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A35)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D35" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A35)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A35)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E35" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A35)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A35)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F35" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A35,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A35,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="G35" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A35,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A35,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H35" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A35,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A35,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I35" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A35,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A35,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J35" s="3" t="str">
@@ -2377,35 +2445,35 @@
         <x:v>home</x:v>
       </x:c>
       <x:c r="B36" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A36)</x:f>
-        <x:v>7</x:v>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A36)</x:f>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C36" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A36)</x:f>
-        <x:v>7</x:v>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A36)</x:f>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D36" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A36)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A36)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E36" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A36)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A36)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F36" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A36,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A36,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G36" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A36,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A36,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H36" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A36,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A36,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I36" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A36,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A36,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="J36" s="3" t="str">
@@ -2421,35 +2489,35 @@
         <x:v>home-cli</x:v>
       </x:c>
       <x:c r="B37" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A37)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A37)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C37" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A37)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A37)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D37" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A37)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A37)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="E37" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A37)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A37)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F37" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A37,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A37,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="G37" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A37,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A37,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H37" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A37,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A37,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I37" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A37,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A37,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="J37" s="3" t="str">
@@ -2465,35 +2533,35 @@
         <x:v>home-gui</x:v>
       </x:c>
       <x:c r="B38" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A38)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A38)</x:f>
         <x:v>16</x:v>
       </x:c>
       <x:c r="C38" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A38)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A38)</x:f>
         <x:v>16</x:v>
       </x:c>
       <x:c r="D38" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A38)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A38)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="E38" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A38)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A38)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="F38" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A38,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A38,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="G38" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A38,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A38,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="H38" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A38,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A38,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I38" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A38,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A38,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="J38" s="3" t="str">
@@ -2509,35 +2577,35 @@
         <x:v>inbox</x:v>
       </x:c>
       <x:c r="B39" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A39)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A39)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="C39" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A39)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A39)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="D39" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A39)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A39)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="E39" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A39)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A39)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F39" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A39,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A39,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G39" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A39,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A39,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="H39" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A39,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A39,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I39" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A39,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A39,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="J39" s="3" t="str">
@@ -2553,35 +2621,35 @@
         <x:v>library</x:v>
       </x:c>
       <x:c r="B40" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A40)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A40)</x:f>
         <x:v>24</x:v>
       </x:c>
       <x:c r="C40" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A40)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A40)</x:f>
         <x:v>23</x:v>
       </x:c>
       <x:c r="D40" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A40)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A40)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="E40" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A40)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A40)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="F40" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A40,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A40,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="G40" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A40,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A40,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="H40" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A40,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A40,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I40" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A40,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A40,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="J40" s="3" t="str">
@@ -2597,35 +2665,35 @@
         <x:v>marketplace</x:v>
       </x:c>
       <x:c r="B41" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A41)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A41)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="C41" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A41)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A41)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D41" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A41)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A41)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E41" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A41)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A41)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="F41" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A41,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A41,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="G41" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A41,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A41,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="H41" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A41,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A41,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I41" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A41,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A41,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="J41" s="3" t="str">
@@ -2641,35 +2709,35 @@
         <x:v>people</x:v>
       </x:c>
       <x:c r="B42" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A42)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A42)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="C42" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A42)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A42)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D42" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A42)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A42)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="E42" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A42)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A42)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F42" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A42,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A42,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G42" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A42,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A42,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="H42" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A42,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A42,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I42" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A42,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A42,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="J42" s="3" t="str">
@@ -2685,35 +2753,35 @@
         <x:v>services</x:v>
       </x:c>
       <x:c r="B43" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A43)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A43)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="C43" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A43)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A43)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D43" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A43)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A43)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="E43" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A43)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A43)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F43" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A43,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A43,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G43" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A43,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A43,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="H43" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A43,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A43,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I43" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A43,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A43,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="J43" s="3" t="str">
@@ -2729,35 +2797,35 @@
         <x:v>system</x:v>
       </x:c>
       <x:c r="B44" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A44)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A44)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="C44" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A44)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A44)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="D44" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A44)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A44)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E44" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A44)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A44)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="F44" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A44,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A44,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="G44" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A44,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A44,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="H44" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A44,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A44,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I44" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A44,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A44,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="J44" s="3" t="str">
@@ -2773,35 +2841,35 @@
         <x:v>wallet</x:v>
       </x:c>
       <x:c r="B45" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A45)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A45)</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="C45" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A45)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A45)</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="D45" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A45)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A45)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="E45" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A45)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A45)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F45" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A45,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A45,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G45" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A45,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A45,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="H45" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A45,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A45,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I45" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A45,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A45,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="J45" s="3" t="str">
@@ -2817,35 +2885,35 @@
         <x:v>wallet-metamask</x:v>
       </x:c>
       <x:c r="B46" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A46)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A46)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C46" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A46)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A46)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D46" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A46)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A46)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E46" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A46)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A46)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F46" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A46,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A46,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G46" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A46,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A46,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H46" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A46,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A46,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I46" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A46,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A46,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="J46" s="3" t="str">
@@ -2861,35 +2929,35 @@
         <x:v>wallet-unisat</x:v>
       </x:c>
       <x:c r="B47" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A47)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A47)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C47" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A47)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A47)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D47" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A47)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A47)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E47" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A47)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A47)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F47" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A47,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A47,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G47" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A47,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A47,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H47" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A47,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A47,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I47" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A47,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A47,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="J47" s="3" t="str">
@@ -2905,35 +2973,35 @@
         <x:v>wallet-walletconnect</x:v>
       </x:c>
       <x:c r="B48" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A48)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A48)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C48" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A48)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A48)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D48" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A48)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A48)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E48" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A48)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A48)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F48" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A48,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A48,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G48" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A48,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A48,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H48" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A48,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A48,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I48" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A48,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A48,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="J48" s="3" t="str">
@@ -2949,35 +3017,35 @@
         <x:v>model-provider</x:v>
       </x:c>
       <x:c r="B49" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A49)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A49)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="C49" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A49)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A49)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D49" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A49)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A49)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E49" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A49)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A49)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F49" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A49,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A49,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G49" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A49,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A49,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H49" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A49,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A49,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I49" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A49,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A49,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="J49" s="3" t="str">
@@ -2993,35 +3061,35 @@
         <x:v>runtime-services</x:v>
       </x:c>
       <x:c r="B50" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A50)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A50)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="C50" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A50)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A50)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D50" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A50)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A50)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E50" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A50)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A50)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F50" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A50,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A50,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="G50" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A50,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A50,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="H50" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A50,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A50,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I50" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A50,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A50,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="J50" s="3" t="str">
@@ -3037,35 +3105,35 @@
         <x:v>shared</x:v>
       </x:c>
       <x:c r="B51" s="14" t="n">
-        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$201,A51)</x:f>
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A51)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C51" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$201,'Journey Matrix'!$P$7:$P$201,A51)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A51)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D51" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$201,'Journey Matrix'!$P$7:$P$201,A51)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A51)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="E51" s="14" t="n">
-        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$201,'Journey Matrix'!$P$7:$P$201,A51)</x:f>
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A51)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F51" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A51,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$8)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A51,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="G51" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A51,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$9)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A51,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H51" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A51,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$11)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A51,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I51" s="14" t="n">
-        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$201,A51,'Journey Matrix'!$D$7:$D$201,'Read Me + Evidence'!$H$10)</x:f>
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A51,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J51" s="3" t="str">
@@ -3076,18 +3144,49 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="52">
-      <x:c r="A52" s="3"/>
-      <x:c r="B52" s="3"/>
-      <x:c r="C52" s="3"/>
-      <x:c r="D52" s="3"/>
-      <x:c r="E52" s="3"/>
-      <x:c r="F52" s="3"/>
-      <x:c r="G52" s="3"/>
-      <x:c r="H52" s="3"/>
-      <x:c r="I52" s="3"/>
-      <x:c r="J52" s="3"/>
-      <x:c r="K52" s="3"/>
+    <x:row r="52" ht="25.5" customHeight="1">
+      <x:c r="A52" s="3" t="str">
+        <x:v>website</x:v>
+      </x:c>
+      <x:c r="B52" s="3" t="n">
+        <x:f>COUNTIF('Journey Matrix'!$P$7:$P$204,A52)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C52" s="3" t="n">
+        <x:f>SUMIFS('Journey Matrix'!$T$7:$T$204,'Journey Matrix'!$P$7:$P$204,A52)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D52" s="3" t="n">
+        <x:f>SUMIFS('Journey Matrix'!$R$7:$R$204,'Journey Matrix'!$P$7:$P$204,A52)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E52" s="3" t="n">
+        <x:f>SUMIFS('Journey Matrix'!$S$7:$S$204,'Journey Matrix'!$P$7:$P$204,A52)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F52" s="3" t="n">
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A52,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$8)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G52" s="3" t="n">
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A52,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$9)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H52" s="3" t="n">
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A52,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$11)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I52" s="3" t="n">
+        <x:f>COUNTIFS('Journey Matrix'!$P$7:$P$204,A52,'Journey Matrix'!$D$7:$D$204,'Read Me + Evidence'!$H$10)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J52" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="K52" s="3" t="n">
+        <x:f>COUNTIF('Control Index'!$B$7:$B$255,A52)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3131,7 +3230,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50c9a5ba1c38444f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbd83dd80bfd49df"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3653,7 +3752,7 @@
         <x:v>Blocked prerequisite</x:v>
       </x:c>
       <x:c r="E11" s="3" t="str">
-        <x:v>Session authority ends and app frames cannot retain privileged access.</x:v>
+        <x:v>Sign-out ends session authority and returns to signed-out /home/. Relock protects Home. Prior app frames retain no privileged access.</x:v>
       </x:c>
       <x:c r="F11" s="12" t="str">
         <x:v>Sign-out/relock would end the shared authenticated Home session. A disposable sign-in target is required; existing user tabs stay authenticated.</x:v>
@@ -3670,10 +3769,12 @@
       <x:c r="J11" s="3" t="str">
         <x:v>1. Save disposable work
 2. Sign out
-3. Revisit prior frame</x:v>
+3. Confirm signed-out /home/
+4. Revisit prior frame and check denied access
+5. Repeat relock separately</x:v>
       </x:c>
       <x:c r="K11" s="3" t="str">
-        <x:v>Disposable signed-in session</x:v>
+        <x:v>Disposable signed-in session; user-controlled passkey; matching installed Home and Runtime receipt</x:v>
       </x:c>
       <x:c r="L11" s="3" t="str"/>
       <x:c r="M11" s="3" t="str"/>
@@ -3702,7 +3803,9 @@
         <x:f>IF(AND(Q11='Read Me + Evidence'!$K$11,D11&lt;&gt;'Read Me + Evidence'!$H$12),1,0)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="U11" s="3" t="str"/>
+      <x:c r="U11" s="3" t="str">
+        <x:v>R2, 2026-09-10: canonical Home entry is /home/. Existing live verdict and evidence remain historical. Repeat sign-out/relock on the exact installed candidate.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="153" customHeight="1">
       <x:c r="A12" s="3" t="str">
@@ -15455,7 +15558,7 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="E192" s="3" t="str">
-        <x:v>Shell exit returns to Desktop; sign-out ends authenticated browser Home session.</x:v>
+        <x:v>Shell exit returns to Desktop. Sign-out ends the authenticated Home session and returns to signed-out /home/.</x:v>
       </x:c>
       <x:c r="F192" s="12" t="str">
         <x:v>Installed b233d832 direct Desktop–Terminal switching and Inbox→Desktop handoff still stall (F44). Reload restores the signed-in selected shell. Native startup, context and repaired Inbox label pass separately. Debugger-independent switching and sign-out remain unverified.</x:v>
@@ -15470,8 +15573,10 @@
         <x:v>q/Esc; exit; signout</x:v>
       </x:c>
       <x:c r="J192" s="3" t="str">
-        <x:v>1. Return to GUI
-2. Inspect separate sign-out action</x:v>
+        <x:v>1. Return to Desktop with q/Esc
+2. Save disposable work
+3. Use the separate sign-out action
+4. Confirm signed-out /home/ and denied prior-frame access</x:v>
       </x:c>
       <x:c r="K192" s="3" t="str">
         <x:v>Disposable shell/session</x:v>
@@ -15505,7 +15610,9 @@
         <x:f>IF(AND(Q192='Read Me + Evidence'!$K$11,D192&lt;&gt;'Read Me + Evidence'!$H$12),1,0)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="U192" s="3" t="str"/>
+      <x:c r="U192" s="3" t="str">
+        <x:v>R2, 2026-09-10: sign-out now names /home/. The existing Fail verdict, F-44/F-53 dispositions and installed evidence stay unchanged until their required proof passes.</x:v>
+      </x:c>
     </x:row>
     <x:row r="193" ht="153" customHeight="1">
       <x:c r="A193" s="3" t="str">
@@ -16081,6 +16188,206 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="U201" s="3" t="str"/>
+    </x:row>
+    <x:row r="202" ht="153" customHeight="1">
+      <x:c r="A202" s="3" t="str">
+        <x:v>AUTH-11</x:v>
+      </x:c>
+      <x:c r="B202" s="3" t="str">
+        <x:v>Home / entry</x:v>
+      </x:c>
+      <x:c r="C202" s="3" t="str">
+        <x:v>Canonical Home and old bookmarks</x:v>
+      </x:c>
+      <x:c r="D202" s="3" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="E202" s="3" t="str">
+        <x:v>/home redirects to /home/. Old Home roots reach that entry; prior assets remain usable. Both manifest URLs retain installed app id /apps/home/ with /home/ start and scope. Existing installed shortcuts reach usable Home. Runtime keeps capsule and API authority.</x:v>
+      </x:c>
+      <x:c r="F202" s="58" t="str">
+        <x:v>Pending target proof for R2. Route source is under review; the register has no installed verdict for this candidate.</x:v>
+      </x:c>
+      <x:c r="G202" s="3" t="str">
+        <x:v>controlled-session</x:v>
+      </x:c>
+      <x:c r="H202" s="3" t="str">
+        <x:v>implemented-source</x:v>
+      </x:c>
+      <x:c r="I202" s="3" t="str">
+        <x:v>Open Home; old bookmark; reload; ordinary app</x:v>
+      </x:c>
+      <x:c r="J202" s="3" t="str">
+        <x:v>1. Open /home and old Home roots with a harmless query
+2. Check modules and both manifest URLs
+3. Check retained asset URL
+4. Launch an existing installed shortcut
+5. Sign in, open app, check API/events and reload</x:v>
+      </x:c>
+      <x:c r="K202" s="3" t="str">
+        <x:v>Approved target and matching artifact receipt; existing installed shortcut; disposable session; user-controlled sign-in</x:v>
+      </x:c>
+      <x:c r="L202" s="3" t="str"/>
+      <x:c r="M202" s="3" t="str"/>
+      <x:c r="N202" s="3" t="str"/>
+      <x:c r="O202" s="3" t="str">
+        <x:v>docs/EXECUTION.md; elastos/crates/elastos-server/src/api/browser_capsules.rs</x:v>
+      </x:c>
+      <x:c r="P202" s="3" t="str">
+        <x:v>home</x:v>
+      </x:c>
+      <x:c r="Q202" s="3" t="str">
+        <x:f>IF(OR(H202='Read Me + Evidence'!$K$6,H202='Read Me + Evidence'!$K$7,H202='Read Me + Evidence'!$K$8,P202='Read Me + Evidence'!$K$9,P202='Read Me + Evidence'!$K$10),'Read Me + Evidence'!$K$12,'Read Me + Evidence'!$K$11)</x:f>
+        <x:v>GUI</x:v>
+      </x:c>
+      <x:c r="R202" s="14" t="n">
+        <x:f>IF(AND(Q202='Read Me + Evidence'!$K$11,OR(D202='Read Me + Evidence'!$H$7,D202='Read Me + Evidence'!$H$8,D202='Read Me + Evidence'!$H$9)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S202" s="14" t="n">
+        <x:f>IF(AND(Q202='Read Me + Evidence'!$K$11,D202='Read Me + Evidence'!$H$7),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T202" s="14" t="n">
+        <x:f>IF(AND(Q202='Read Me + Evidence'!$K$11,D202&lt;&gt;'Read Me + Evidence'!$H$12),1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U202" s="3" t="str">
+        <x:v>R2, 2026-09-10. C1-home/C1-seed. Installed-shortcut migration needs target proof. Preserve AUTH-04, AUTH-05 and CLI-05 proof boundaries.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="203" ht="153" customHeight="1">
+      <x:c r="A203" s="3" t="str">
+        <x:v>SITE-01</x:v>
+      </x:c>
+      <x:c r="B203" s="3" t="str">
+        <x:v>Public website</x:v>
+      </x:c>
+      <x:c r="C203" s="3" t="str">
+        <x:v>Read storefront and open Home</x:v>
+      </x:c>
+      <x:c r="D203" s="3" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="E203" s="3" t="str">
+        <x:v>The storefront explains available use and keeps hosted Home, source and public download facts distinct. Open Home uses same-origin /home/. Desktop, mobile and keyboard actions remain clear and usable.</x:v>
+      </x:c>
+      <x:c r="F203" s="58" t="str">
+        <x:v>Pending target proof for R2. A source draft or local preview alone does not prove the seed serves this candidate.</x:v>
+      </x:c>
+      <x:c r="G203" s="3" t="str">
+        <x:v>safe-read-only</x:v>
+      </x:c>
+      <x:c r="H203" s="3" t="str">
+        <x:v>implemented-source</x:v>
+      </x:c>
+      <x:c r="I203" s="3" t="str">
+        <x:v>Open Home; source guide; release evidence; keyboard navigation</x:v>
+      </x:c>
+      <x:c r="J203" s="3" t="str">
+        <x:v>1. Open the public root at desktop and mobile widths
+2. Use keyboard focus and links
+3. Select Open Home and confirm same-origin /home/
+4. Follow the source guide and release evidence links</x:v>
+      </x:c>
+      <x:c r="K203" s="3" t="str">
+        <x:v>Reviewed site on approved target; served artifact receipt; desktop/mobile browser and keyboard; public Home entry</x:v>
+      </x:c>
+      <x:c r="L203" s="3" t="str"/>
+      <x:c r="M203" s="3" t="str"/>
+      <x:c r="N203" s="3" t="str"/>
+      <x:c r="O203" s="3" t="str">
+        <x:v>docs/EXECUTION.md; website/elastos/index.html; website/elastos/site.mjs</x:v>
+      </x:c>
+      <x:c r="P203" s="3" t="str">
+        <x:v>website</x:v>
+      </x:c>
+      <x:c r="Q203" s="3" t="str">
+        <x:f>IF(OR(H203='Read Me + Evidence'!$K$6,H203='Read Me + Evidence'!$K$7,H203='Read Me + Evidence'!$K$8,P203='Read Me + Evidence'!$K$9,P203='Read Me + Evidence'!$K$10),'Read Me + Evidence'!$K$12,'Read Me + Evidence'!$K$11)</x:f>
+        <x:v>GUI</x:v>
+      </x:c>
+      <x:c r="R203" s="14" t="n">
+        <x:f>IF(AND(Q203='Read Me + Evidence'!$K$11,OR(D203='Read Me + Evidence'!$H$7,D203='Read Me + Evidence'!$H$8,D203='Read Me + Evidence'!$H$9)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S203" s="14" t="n">
+        <x:f>IF(AND(Q203='Read Me + Evidence'!$K$11,D203='Read Me + Evidence'!$H$7),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T203" s="14" t="n">
+        <x:f>IF(AND(Q203='Read Me + Evidence'!$K$11,D203&lt;&gt;'Read Me + Evidence'!$H$12),1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U203" s="3" t="str">
+        <x:v>R2, 2026-09-10. C1-site/C1-seed. Full release and installer acceptance stay in J1-J5/C6.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204" ht="153" customHeight="1">
+      <x:c r="A204" s="3" t="str">
+        <x:v>SITE-02</x:v>
+      </x:c>
+      <x:c r="B204" s="3" t="str">
+        <x:v>Public website</x:v>
+      </x:c>
+      <x:c r="C204" s="3" t="str">
+        <x:v>Installer metadata and failure states</x:v>
+      </x:c>
+      <x:c r="D204" s="3" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="E204" s="3" t="str">
+        <x:v>Installer availability needs matching release facts, the selected platform and its recorded install proof. Missing, malformed, inconsistent or unsupported data leaves an honest usable action. A displayed SHA-256 is a checksum; installer signature verification has its own claim.</x:v>
+      </x:c>
+      <x:c r="F204" s="58" t="str">
+        <x:v>Pending target proof for R2. Controlled metadata responses must be observed through the rendered page before a live verdict.</x:v>
+      </x:c>
+      <x:c r="G204" s="3" t="str">
+        <x:v>safe-read-only</x:v>
+      </x:c>
+      <x:c r="H204" s="3" t="str">
+        <x:v>implemented-source</x:v>
+      </x:c>
+      <x:c r="I204" s="3" t="str">
+        <x:v>Platform selector; installer action; source guide; metadata and checksum</x:v>
+      </x:c>
+      <x:c r="J204" s="3" t="str">
+        <x:v>1. Inspect matching release/platform with and without install proof
+2. Select an unsupported platform
+3. Exercise missing, malformed and mismatched metadata
+4. Confirm unavailable installer action and usable source/Home links
+5. Check checksum wording</x:v>
+      </x:c>
+      <x:c r="K204" s="3" t="str">
+        <x:v>Isolated response fixtures on the reviewed page; approved target smoke with its real metadata; avoid changing the public publisher</x:v>
+      </x:c>
+      <x:c r="L204" s="3" t="str"/>
+      <x:c r="M204" s="3" t="str"/>
+      <x:c r="N204" s="3" t="str"/>
+      <x:c r="O204" s="3" t="str">
+        <x:v>docs/EXECUTION.md; website/elastos/site.mjs; website/elastos/claims.json</x:v>
+      </x:c>
+      <x:c r="P204" s="3" t="str">
+        <x:v>website</x:v>
+      </x:c>
+      <x:c r="Q204" s="3" t="str">
+        <x:f>IF(OR(H204='Read Me + Evidence'!$K$6,H204='Read Me + Evidence'!$K$7,H204='Read Me + Evidence'!$K$8,P204='Read Me + Evidence'!$K$9,P204='Read Me + Evidence'!$K$10),'Read Me + Evidence'!$K$12,'Read Me + Evidence'!$K$11)</x:f>
+        <x:v>GUI</x:v>
+      </x:c>
+      <x:c r="R204" s="14" t="n">
+        <x:f>IF(AND(Q204='Read Me + Evidence'!$K$11,OR(D204='Read Me + Evidence'!$H$7,D204='Read Me + Evidence'!$H$8,D204='Read Me + Evidence'!$H$9)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S204" s="14" t="n">
+        <x:f>IF(AND(Q204='Read Me + Evidence'!$K$11,D204='Read Me + Evidence'!$H$7),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T204" s="14" t="n">
+        <x:f>IF(AND(Q204='Read Me + Evidence'!$K$11,D204&lt;&gt;'Read Me + Evidence'!$H$12),1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U204" s="3" t="str">
+        <x:v>R2, 2026-09-10. C1-site/C1-proof. Fixtures prove page behavior; record real served metadata and installer acceptance separately.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -16107,14 +16414,37 @@
       <x:formula>"Not run"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="1">
+  <x:conditionalFormatting sqref="D202:D204">
+    <x:cfRule type="cellIs" dxfId="37" priority="7" operator="equal">
+      <x:formula>"Pass"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="38" priority="8" operator="equal">
+      <x:formula>"Fail"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="39" priority="9" operator="equal">
+      <x:formula>"Partially observed"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="40" priority="10" operator="equal">
+      <x:formula>"Blocked prerequisite"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="41" priority="11" operator="equal">
+      <x:formula>"Blocked tool"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="42" priority="12" operator="equal">
+      <x:formula>"Not run"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="D7:D201">
+      <x:formula1>"Not run,Pass,Fail,Partially observed,Blocked prerequisite,Blocked tool,Not applicable"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D202:D204">
       <x:formula1>"Not run,Pass,Fail,Partially observed,Blocked prerequisite,Blocked tool,Not applicable"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R562c5740ef324d73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0dbeacf9bbe4b87"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27775,8 +28105,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7017081ee9e147bb"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d7f30e34d784a20"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35a34facaec94985"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c2f776b02f847fb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30287,7 +30617,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d6ceee7dd914057"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1bd54ba27e3849cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32414,7 +32744,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14d89847794342f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5c8594e64cb47d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40721,7 +41051,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc35b5f9d21b945a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recef94be20804f93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -43683,7 +44013,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb003a05f3a641cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb72d2226f11342bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record restored Home user-review repairs and proof
</commit_message>
<xml_diff>
--- a/docs/audits/ElastOS-Home-Journey-Audit.xlsx
+++ b/docs/audits/ElastOS-Home-Journey-Audit.xlsx
@@ -3496,8 +3496,10 @@
           <x:t xml:space="preserve">Create stores the protected Profile and name before exporting a complete Recovery Kit. Recover selects a kit first, then sets up a passkey and restores the original Profile DID and exact name.</x:t>
         </x:is>
       </x:c>
-      <x:c r="F7" s="12" t="str">
-        <x:v>Creating a first account needs a fresh target and a user-operated passkey. Existing accounts and passkeys were preserved.</x:v>
+      <x:c r="F7" s="12" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">User review exercised recovery in both isolated Homes and reported an unnamed account label and cross-port session conflict. Candidate 1e320578 repairs both; automated installed proof passes. Final user confirmation of original Profile DID/name remains pending; AUTH-01 verdict stays unchanged.</x:t>
+        </x:is>
       </x:c>
       <x:c r="G7" s="3" t="str">
         <x:v>controlled-identity</x:v>
@@ -3569,8 +3571,10 @@
       <x:c r="E8" s="3" t="str">
         <x:v>Valid passkey opens that principal's shell; cancellation leaves Home locked.</x:v>
       </x:c>
-      <x:c r="F8" s="12" t="str">
-        <x:v>Brave resumes the existing authenticated session. A fresh passkey sign-in was not forced because it would disturb the current session.</x:v>
+      <x:c r="F8" s="12" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Candidate 1e320578: one Brave context keeps Mac and Linux localhost Homes signed in through alternating cookie-only reloads and refreshes. Virtual CTAP2 evidence; final user acceptance remains pending. Legacy unscoped cookie-only sessions need one sign-in after upgrade.</x:t>
+        </x:is>
       </x:c>
       <x:c r="G8" s="3" t="str">
         <x:v>controlled-identity</x:v>
@@ -3762,8 +3766,10 @@
       <x:c r="E11" s="3" t="str">
         <x:v>Sign-out ends session authority and returns to signed-out /home/. Relock protects Home. Prior app frames retain no privileged access.</x:v>
       </x:c>
-      <x:c r="F11" s="12" t="str">
-        <x:v>Sign-out/relock would end the shared authenticated Home session. A disposable sign-in target is required; existing user tabs stay authenticated.</x:v>
+      <x:c r="F11" s="12" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Candidate 1e320578: signing out of Mac clears only its destination-scoped cookie and leaves Linux signed in through reload and refresh. Existing strict session authority checks pass. Relock and other listed branches retain their prior scope.</x:t>
+        </x:is>
       </x:c>
       <x:c r="G11" s="3" t="str">
         <x:v>controlled-session</x:v>
@@ -5153,8 +5159,10 @@
       <x:c r="E32" s="3" t="str">
         <x:v>Current account/role are clear. Runtime authorizes sensitive changes and protects account ownership.</x:v>
       </x:c>
-      <x:c r="F32" s="12" t="str">
-        <x:v>Accounts shows the existing current passkey account and role. Role/removal dispatch is excluded to preserve ownership; disposable-account authorization required for remaining branches.</x:v>
+      <x:c r="F32" s="12" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Candidate 1e320578: installed Mac and Linux foreground Accounts display the exact restored Profile name for the current unnamed passkey. Explicit private labels remain intact; another account never borrows that Profile name. Role/removal acceptance retains its prior scope.</x:t>
+        </x:is>
       </x:c>
       <x:c r="G32" s="3" t="str">
         <x:v>controlled-identity</x:v>
@@ -5804,8 +5812,10 @@
       <x:c r="E42" s="3" t="str">
         <x:v>Runtime projects exact scope and approval; descriptors are not grants.</x:v>
       </x:c>
-      <x:c r="F42" s="12" t="str">
-        <x:v>Technical Details expands and lists49objects. Archive Manager is selected with bounded identifier/author/type/role/version and explicit Unverified status. Operator effect preview/approval remains untested; no request dispatched. E103 independently verifies read-only Refresh and unchanged inventory.</x:v>
+      <x:c r="F42" s="12" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Candidate 1e320578 adds space around the Advanced object count and Refresh toolbar. Rendered 980px/420px checks and installed source/served parity pass. Prior technical inspection and approval evidence retains its exact scope.</x:t>
+        </x:is>
       </x:c>
       <x:c r="G42" s="3" t="str">
         <x:v>privileged-operator</x:v>

</xml_diff>